<commit_message>
New Map view built with Leaflet, 05-Maps sample report
One point per row of the model (latitude / longitude columns found by name),
color and size columns, legend, popup with the navigation links, background
maps OpenStreetMap, OpenTopoMap, OpenHikingMap, IGN Plan or custom tiles.
The column parameters of the view follow the elements changed by a drill navigation.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D496"/>
+  <dimension ref="A1:D498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9379,6 +9379,40 @@
         </is>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>{0} point(s) displayed</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>{0} point(s) affiché(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>{0} row(s) without coordinates</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>{0} ligne(s) sans coordonnées</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Reset restrictions button: restore the initial prompted restriction values without executing the report
- ReportExecution saves the prompted restriction values before the first user input and
  ResetPromptedRestrictions() restores them and re-renders the restrictions panel
- ActionResetRestrictions (web) / ResetRestrictions (Designer viewer)
- Header button next to Show Restrictions (report header + web menu), translations
- 05-Maps sample: more default countries; IIS Express SSL port 44310 (44398 reserved by Windows)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D498"/>
+  <dimension ref="A1:D499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9413,6 +9413,23 @@
         </is>
       </c>
     </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Reset restrictions</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Réinitialiser les restrictions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
AI chat: no Execute button for a report that does not exist
- SWIGetAIAgentResponse drops an [EXECUTE_REPORT:...] button whose .srex is not found,
  logs a warning and appends a translated note (the model may announce a report it never created).
- build-report-from-metadata / build-report-from-sql skills: a report exists only once the
  create tool has returned success in the current turn.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D499"/>
+  <dimension ref="A1:D500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9430,6 +9430,23 @@
         </is>
       </c>
     </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>The report '{0}' was not found: it has not been created or it was moved.</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Le rapport '{0}' est introuvable : il n'a pas été créé ou il a été déplacé.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Data Entry module: ignore the deployed DataTableEditor views, French translations of the editor messages
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D500"/>
+  <dimension ref="A1:D520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9447,6 +9447,346 @@
         </is>
       </c>
     </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>This key already exists</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Cette clé existe déjà</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>A record with the same key or unique value already exists</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Un enregistrement avec la même clé ou valeur unique existe déjà</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Record not found</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Enregistrement introuvable</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>This operation is not allowed</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Cette opération n'est pas autorisée</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>No record has been modified</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Aucun enregistrement n'a été modifié</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Invalid value</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Valeur invalide</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>An error occurred</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Une erreur s'est produite</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Unable to reach the server</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Impossible de joindre le serveur</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Your session has expired, please reload the page</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Votre session a expiré, veuillez recharger la page</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Are you sure you want to delete this record?</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Voulez-vous vraiment supprimer cet enregistrement ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Edit record</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Modifier l'enregistrement</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>New record</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Nouvel enregistrement</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>The record has been created</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>L'enregistrement a été créé</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>The record has been deleted</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>L'enregistrement a été supprimé</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>The record has been saved</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>L'enregistrement a été enregistré</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>The table cannot be edited here</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>La table ne peut pas être modifiée ici</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Supprimer</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Modifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Enregistrer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Web login dialogs: standard card layout for login, two-factor, password reset and change (centered 400px card, icon badge header, real forms with autocomplete, show/hide password, inline errors, signed-out message); Back to login links fixed; failed login no longer reveals the previous folders and reports
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D520"/>
+  <dimension ref="A1:D523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9787,6 +9787,57 @@
         </is>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>You have been signed out.</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Vous avez été déconnecté.</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Show password</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Afficher le mot de passe</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>or</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>ou</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Web schedules: file name of the output edited with an editable combo (as in eReports) proposing the report display name keyword or the report name, with or without the execution date time ({0:yyyy_MM_dd}, {0:yyyy_MM_dd HH_mm_ss}); the format of the execution date in the file name is checked when the schedule is saved; System report '320 Reports - Server Schedule Definitions': the web schedules of all the users are listed with the schedules of their report (output 'Web schedule of <user>'), the report of a web schedule not found in the scanned folders (e.g. personal folder of another user) is loaded from the schedule; French translations; swi-schedule.min.js regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D652"/>
+  <dimension ref="A1:D654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12031,6 +12031,40 @@
         </is>
       </c>
     </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>File names with the execution date time</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Noms de fichier avec la date et l'heure d'exécution</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>The format of the execution date in the file name is invalid</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Le format de la date d'exécution dans le nom du fichier est invalide</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>